<commit_message>
estandariza nombres de carpetas de distritos segun Excel de referencia
- renombra 8 carpetas en datos/ para coincidir exactamente con
  nombre_distrito_estandarizado (sin underscores, minusculas, sin tildes):
  san_bernardino→sanbernardino, fernando_de_la_mora→fernandodelamora,
  mariano_roque_alonso→marianoroquealonso, ja_saldivar→joseaugustosaldivar,
  nueva_italia→nuevaitalia, villa_elisa→villaelisa,
  san_antonio→sanantonio, san_lorenzo→sanlorenzo
- actualiza progreso.xlsx (96 celdas corregidas)
- agrega seccion en manual sobre nombres de carpetas con referencia al
  archivo nombres_estandarizados_distritos_PRY.xlsx
- agrega nombres_estandarizados_distritos_PRY.xlsx en manual/

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/registro_progreso/progreso.xlsx
+++ b/registro_progreso/progreso.xlsx
@@ -2189,7 +2189,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>fernando_de_la_mora</t>
+          <t>fernandodelamora</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>fernando_de_la_mora</t>
+          <t>fernandodelamora</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>fernando_de_la_mora</t>
+          <t>fernandodelamora</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>fernando_de_la_mora</t>
+          <t>fernandodelamora</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>fernando_de_la_mora</t>
+          <t>fernandodelamora</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>fernando_de_la_mora</t>
+          <t>fernandodelamora</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>fernando_de_la_mora</t>
+          <t>fernandodelamora</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>fernando_de_la_mora</t>
+          <t>fernandodelamora</t>
         </is>
       </c>
       <c r="C45" s="3" t="n">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>fernando_de_la_mora</t>
+          <t>fernandodelamora</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>fernando_de_la_mora</t>
+          <t>fernandodelamora</t>
         </is>
       </c>
       <c r="C47" s="3" t="n">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>fernando_de_la_mora</t>
+          <t>fernandodelamora</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>fernando_de_la_mora</t>
+          <t>fernandodelamora</t>
         </is>
       </c>
       <c r="C49" s="3" t="n">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>san_lorenzo</t>
+          <t>sanlorenzo</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>san_lorenzo</t>
+          <t>sanlorenzo</t>
         </is>
       </c>
       <c r="C51" s="3" t="n">
@@ -2833,7 +2833,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>san_lorenzo</t>
+          <t>sanlorenzo</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>san_lorenzo</t>
+          <t>sanlorenzo</t>
         </is>
       </c>
       <c r="C53" s="3" t="n">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>san_lorenzo</t>
+          <t>sanlorenzo</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>san_lorenzo</t>
+          <t>sanlorenzo</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
@@ -3017,7 +3017,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>san_lorenzo</t>
+          <t>sanlorenzo</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3063,7 +3063,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>san_lorenzo</t>
+          <t>sanlorenzo</t>
         </is>
       </c>
       <c r="C57" s="3" t="n">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>san_lorenzo</t>
+          <t>sanlorenzo</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>san_lorenzo</t>
+          <t>sanlorenzo</t>
         </is>
       </c>
       <c r="C59" s="3" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>san_lorenzo</t>
+          <t>sanlorenzo</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -3247,7 +3247,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>san_lorenzo</t>
+          <t>sanlorenzo</t>
         </is>
       </c>
       <c r="C61" s="3" t="n">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>mariano_roque_alonso</t>
+          <t>marianoroquealonso</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -4995,7 +4995,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>mariano_roque_alonso</t>
+          <t>marianoroquealonso</t>
         </is>
       </c>
       <c r="C99" s="3" t="n">
@@ -5041,7 +5041,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>mariano_roque_alonso</t>
+          <t>marianoroquealonso</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>mariano_roque_alonso</t>
+          <t>marianoroquealonso</t>
         </is>
       </c>
       <c r="C101" s="3" t="n">
@@ -5133,7 +5133,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>mariano_roque_alonso</t>
+          <t>marianoroquealonso</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>mariano_roque_alonso</t>
+          <t>marianoroquealonso</t>
         </is>
       </c>
       <c r="C103" s="3" t="n">
@@ -5225,7 +5225,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>mariano_roque_alonso</t>
+          <t>marianoroquealonso</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>mariano_roque_alonso</t>
+          <t>marianoroquealonso</t>
         </is>
       </c>
       <c r="C105" s="3" t="n">
@@ -5317,7 +5317,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>mariano_roque_alonso</t>
+          <t>marianoroquealonso</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>mariano_roque_alonso</t>
+          <t>marianoroquealonso</t>
         </is>
       </c>
       <c r="C107" s="3" t="n">
@@ -5409,7 +5409,7 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>mariano_roque_alonso</t>
+          <t>marianoroquealonso</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -5455,7 +5455,7 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>mariano_roque_alonso</t>
+          <t>marianoroquealonso</t>
         </is>
       </c>
       <c r="C109" s="3" t="n">
@@ -6053,7 +6053,7 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>ja_saldivar</t>
+          <t>joseaugustosaldivar</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>ja_saldivar</t>
+          <t>joseaugustosaldivar</t>
         </is>
       </c>
       <c r="C123" s="3" t="n">
@@ -6145,7 +6145,7 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>ja_saldivar</t>
+          <t>joseaugustosaldivar</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
@@ -6191,7 +6191,7 @@
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>ja_saldivar</t>
+          <t>joseaugustosaldivar</t>
         </is>
       </c>
       <c r="C125" s="3" t="n">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>ja_saldivar</t>
+          <t>joseaugustosaldivar</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>ja_saldivar</t>
+          <t>joseaugustosaldivar</t>
         </is>
       </c>
       <c r="C127" s="3" t="n">
@@ -6329,7 +6329,7 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>ja_saldivar</t>
+          <t>joseaugustosaldivar</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
@@ -6375,7 +6375,7 @@
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>ja_saldivar</t>
+          <t>joseaugustosaldivar</t>
         </is>
       </c>
       <c r="C129" s="3" t="n">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>ja_saldivar</t>
+          <t>joseaugustosaldivar</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
@@ -6467,7 +6467,7 @@
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>ja_saldivar</t>
+          <t>joseaugustosaldivar</t>
         </is>
       </c>
       <c r="C131" s="3" t="n">
@@ -6513,7 +6513,7 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>ja_saldivar</t>
+          <t>joseaugustosaldivar</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
@@ -6559,7 +6559,7 @@
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>ja_saldivar</t>
+          <t>joseaugustosaldivar</t>
         </is>
       </c>
       <c r="C133" s="3" t="n">
@@ -7157,7 +7157,7 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>villa_elisa</t>
+          <t>villaelisa</t>
         </is>
       </c>
       <c r="C146" s="2" t="n">
@@ -7203,7 +7203,7 @@
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>villa_elisa</t>
+          <t>villaelisa</t>
         </is>
       </c>
       <c r="C147" s="3" t="n">
@@ -7249,7 +7249,7 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>villa_elisa</t>
+          <t>villaelisa</t>
         </is>
       </c>
       <c r="C148" s="2" t="n">
@@ -7295,7 +7295,7 @@
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>villa_elisa</t>
+          <t>villaelisa</t>
         </is>
       </c>
       <c r="C149" s="3" t="n">
@@ -7341,7 +7341,7 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>villa_elisa</t>
+          <t>villaelisa</t>
         </is>
       </c>
       <c r="C150" s="2" t="n">
@@ -7387,7 +7387,7 @@
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>villa_elisa</t>
+          <t>villaelisa</t>
         </is>
       </c>
       <c r="C151" s="3" t="n">
@@ -7433,7 +7433,7 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>villa_elisa</t>
+          <t>villaelisa</t>
         </is>
       </c>
       <c r="C152" s="2" t="n">
@@ -7479,7 +7479,7 @@
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>villa_elisa</t>
+          <t>villaelisa</t>
         </is>
       </c>
       <c r="C153" s="3" t="n">
@@ -7525,7 +7525,7 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>villa_elisa</t>
+          <t>villaelisa</t>
         </is>
       </c>
       <c r="C154" s="2" t="n">
@@ -7571,7 +7571,7 @@
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>villa_elisa</t>
+          <t>villaelisa</t>
         </is>
       </c>
       <c r="C155" s="3" t="n">
@@ -7617,7 +7617,7 @@
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>villa_elisa</t>
+          <t>villaelisa</t>
         </is>
       </c>
       <c r="C156" s="2" t="n">
@@ -7663,7 +7663,7 @@
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>villa_elisa</t>
+          <t>villaelisa</t>
         </is>
       </c>
       <c r="C157" s="3" t="n">
@@ -7709,7 +7709,7 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>san_antonio</t>
+          <t>sanantonio</t>
         </is>
       </c>
       <c r="C158" s="2" t="n">
@@ -7755,7 +7755,7 @@
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>san_antonio</t>
+          <t>sanantonio</t>
         </is>
       </c>
       <c r="C159" s="3" t="n">
@@ -7801,7 +7801,7 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>san_antonio</t>
+          <t>sanantonio</t>
         </is>
       </c>
       <c r="C160" s="2" t="n">
@@ -7847,7 +7847,7 @@
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>san_antonio</t>
+          <t>sanantonio</t>
         </is>
       </c>
       <c r="C161" s="3" t="n">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>san_antonio</t>
+          <t>sanantonio</t>
         </is>
       </c>
       <c r="C162" s="2" t="n">
@@ -7939,7 +7939,7 @@
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>san_antonio</t>
+          <t>sanantonio</t>
         </is>
       </c>
       <c r="C163" s="3" t="n">
@@ -7985,7 +7985,7 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>san_antonio</t>
+          <t>sanantonio</t>
         </is>
       </c>
       <c r="C164" s="2" t="n">
@@ -8031,7 +8031,7 @@
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>san_antonio</t>
+          <t>sanantonio</t>
         </is>
       </c>
       <c r="C165" s="3" t="n">
@@ -8077,7 +8077,7 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>san_antonio</t>
+          <t>sanantonio</t>
         </is>
       </c>
       <c r="C166" s="2" t="n">
@@ -8123,7 +8123,7 @@
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>san_antonio</t>
+          <t>sanantonio</t>
         </is>
       </c>
       <c r="C167" s="3" t="n">
@@ -8169,7 +8169,7 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>san_antonio</t>
+          <t>sanantonio</t>
         </is>
       </c>
       <c r="C168" s="2" t="n">
@@ -8215,7 +8215,7 @@
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>san_antonio</t>
+          <t>sanantonio</t>
         </is>
       </c>
       <c r="C169" s="3" t="n">
@@ -10469,7 +10469,7 @@
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>nueva_italia</t>
+          <t>nuevaitalia</t>
         </is>
       </c>
       <c r="C218" s="2" t="n">
@@ -10515,7 +10515,7 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>nueva_italia</t>
+          <t>nuevaitalia</t>
         </is>
       </c>
       <c r="C219" s="3" t="n">
@@ -10561,7 +10561,7 @@
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>nueva_italia</t>
+          <t>nuevaitalia</t>
         </is>
       </c>
       <c r="C220" s="2" t="n">
@@ -10607,7 +10607,7 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>nueva_italia</t>
+          <t>nuevaitalia</t>
         </is>
       </c>
       <c r="C221" s="3" t="n">
@@ -10653,7 +10653,7 @@
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>nueva_italia</t>
+          <t>nuevaitalia</t>
         </is>
       </c>
       <c r="C222" s="2" t="n">
@@ -10699,7 +10699,7 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>nueva_italia</t>
+          <t>nuevaitalia</t>
         </is>
       </c>
       <c r="C223" s="3" t="n">
@@ -10745,7 +10745,7 @@
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>nueva_italia</t>
+          <t>nuevaitalia</t>
         </is>
       </c>
       <c r="C224" s="2" t="n">
@@ -10791,7 +10791,7 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>nueva_italia</t>
+          <t>nuevaitalia</t>
         </is>
       </c>
       <c r="C225" s="3" t="n">
@@ -10837,7 +10837,7 @@
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t>nueva_italia</t>
+          <t>nuevaitalia</t>
         </is>
       </c>
       <c r="C226" s="2" t="n">
@@ -10883,7 +10883,7 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>nueva_italia</t>
+          <t>nuevaitalia</t>
         </is>
       </c>
       <c r="C227" s="3" t="n">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>nueva_italia</t>
+          <t>nuevaitalia</t>
         </is>
       </c>
       <c r="C228" s="2" t="n">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>nueva_italia</t>
+          <t>nuevaitalia</t>
         </is>
       </c>
       <c r="C229" s="3" t="n">
@@ -11573,7 +11573,7 @@
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>san_bernardino</t>
+          <t>sanbernardino</t>
         </is>
       </c>
       <c r="C242" s="2" t="n">
@@ -11619,7 +11619,7 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>san_bernardino</t>
+          <t>sanbernardino</t>
         </is>
       </c>
       <c r="C243" s="3" t="n">
@@ -11665,7 +11665,7 @@
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>san_bernardino</t>
+          <t>sanbernardino</t>
         </is>
       </c>
       <c r="C244" s="2" t="n">
@@ -11711,7 +11711,7 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>san_bernardino</t>
+          <t>sanbernardino</t>
         </is>
       </c>
       <c r="C245" s="3" t="n">
@@ -11757,7 +11757,7 @@
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>san_bernardino</t>
+          <t>sanbernardino</t>
         </is>
       </c>
       <c r="C246" s="2" t="n">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>san_bernardino</t>
+          <t>sanbernardino</t>
         </is>
       </c>
       <c r="C247" s="3" t="n">
@@ -11849,7 +11849,7 @@
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>san_bernardino</t>
+          <t>sanbernardino</t>
         </is>
       </c>
       <c r="C248" s="2" t="n">
@@ -11895,7 +11895,7 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>san_bernardino</t>
+          <t>sanbernardino</t>
         </is>
       </c>
       <c r="C249" s="3" t="n">
@@ -11941,7 +11941,7 @@
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>san_bernardino</t>
+          <t>sanbernardino</t>
         </is>
       </c>
       <c r="C250" s="2" t="n">
@@ -11987,7 +11987,7 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>san_bernardino</t>
+          <t>sanbernardino</t>
         </is>
       </c>
       <c r="C251" s="3" t="n">
@@ -12033,7 +12033,7 @@
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>san_bernardino</t>
+          <t>sanbernardino</t>
         </is>
       </c>
       <c r="C252" s="2" t="n">
@@ -12079,7 +12079,7 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>san_bernardino</t>
+          <t>sanbernardino</t>
         </is>
       </c>
       <c r="C253" s="3" t="n">

</xml_diff>